<commit_message>
refactor: reclassify by sector relevance per Harkalm acquisition criteria
Rewrite prompt and baseline to classify vacant/former properties in their
sector (Nursery, Food Store) rather than defaulting to None. Update docs
and regenerate results.
</commit_message>
<xml_diff>
--- a/results/listings_classified.xlsx
+++ b/results/listings_classified.xlsx
@@ -26,12 +26,17 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -50,7 +55,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00FCE4EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,12 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,22 +479,22 @@
           <t>HK-F001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Food Store</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>States “former Co‑op convenience store,” “vacant since the operator’s relocation,” and “vacant possession.” Therefore not currently operating as a food store. Former sector use and retained fit-out/suitability language warrant Medium confidence.</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="b">
+          <t>The listing is a former Co-op convenience store with retained food-retail fixtures (chillers, shelving) and is vacant, making it acquisition-relevant as a food retail property. Presence of former/vacant target-sector use triggers Medium confidence per rules.</t>
+        </is>
+      </c>
+      <c r="E2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -503,18 +509,18 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current use is a parcel of ancient woodland/land with no operating business; not a nursery, SEN school, or food store. Listing uses future-use language (“opportunity to build subject to planning”), which signals uncommitted use and triggers Medium confidence per rules.</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="b">
-        <v>1</v>
+          <t>Listing is for an acre of ancient woodland/land with generic development potential; no current or former nursery, SEN school, or food store use or consent indicated. Generic opportunity language does not qualify under the rules.</t>
+        </is>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -528,14 +534,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Currently fully let as generic retail with ancillary storage and an upper-floor dance studio. No indication of a children’s nursery, SEN school, or a food retail store tenant.</t>
+          <t>Property is a fully let mixed-use investment with generic retail on ground/first floors and a dance studio on the second. No indication of current or former use as a nursery, SEN school, or food store, and no suitability/alternative-use language. Therefore not relevant to target sectors.</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -553,17 +559,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Described as a former café; business has ceased trading and the property is offered with vacant possession, so there is no current use in target sectors. Mentions “suitable for”/future uses, which flags uncommitted current use — hence Medium confidence.</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="b">
+          <t>The property is a former café with residential accommodation above and generic ‘variety of alternative uses’ language. There is no indication of current or former use as a nursery, SEN school, or food retail store. Nearby occupiers (e.g., Co-Op) are location context only. Suitability/alternative-use phrasing triggers Medium confidence per rules.</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -578,17 +584,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Described as a former doctor’s surgery with “ideal for” alternative uses, indicating no current operation. No current nursery, SEN school, or food store tenant is stated. Rules 2 and 3 apply.</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="b">
+          <t>The property is a former doctor’s surgery with generic suitability language for various uses. There is no mention of a nursery, SEN school, or food store current or former use. Generic suitability phrases are present, triggering Medium confidence.</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -603,14 +609,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Currently a ground-floor sunbed/tanning shop with a residential flat above. No operation as a nursery, SEN school, or food store. Nearby Budgens/Premier store is a location point and not the subject property.</t>
+          <t>Property comprises a tanning shop with a flat above; no current or former nursery, SEN school, or food store use. Mention of a Budgens/Premier store is merely nearby (location context) and must be ignored per rules.</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -630,16 +636,16 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Currently a mixed-use property: ground/lower floors are a retail shop and workshop selling bath products; upper floors are a holiday apartment. Not a food store, nursery, or SEN school, and no vacancy/“former” language.</t>
+          <t>Mixed-use property with a retail shop (bath products) and a holiday apartment. No indication of current or former use as a nursery, SEN school, or food store. Includes suitability phrasing (“could be used for a new retail business”), triggering Medium confidence per rules.</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -653,14 +659,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Listing is a pub (freehouse/public house) with accommodation; no indication of nursery, SEN school, or food retail current use.</t>
+          <t>Listing is a Grade II listed freehouse pub with accommodation; no mention of nursery, SEN school, or food retail current or former use. Nearby schools are location context only.</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -678,14 +684,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Multi-let industrial/trade park with industrial and trade counter units; no current nursery, SEN school, or food retail operation stated. Nearby occupiers listed are location context only.</t>
+          <t>A fully let multi-let industrial/trade park investment with trade counter units; no current or former nursery, SEN school, or food retail use indicated and no sector-specific fit-out or consent mentioned.</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -703,14 +709,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Currently operates as a fire door manufacturer/joinery business in an industrial property; no current operation as nursery, SEN school, or food store.</t>
+          <t>Industrial business sale for a fire door manufacturer/joinery with no indication of current or former use as a nursery, SEN school, or food store, nor any sector-specific planning or fit-out mentioned.</t>
         </is>
       </c>
       <c r="E11" t="b">
@@ -728,14 +734,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Current uses are a workshop/garage let to an unspecified business and a separate ground-floor retail unit sold off on a long lease; no indication of a nursery, SEN school, or food retail tenant. Mentions of Tesco Express are only as nearby occupiers. Airspace/development potential is irrelevant to current use.</t>
+          <t>The listing is a mixed-use freehold investment comprising a workshop/garage and a separate retail shop sold off on a long lease. No mention of nursery, SEN school, or food retail use for the subject premises; references to Tesco Express are only nearby occupiers and must be ignored. Development/airspace notes do not relate to a target-sector tenant. Therefore, no meaningful connection to Nursery, SEN School, or Food Store.</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -753,17 +759,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Currently marketed as a healthcare/medical premises and described as a blank canvas with flexible terms, indicating no current tenant. Not operating as a nursery, SEN school, or food store. The Co-Op is only a nearby point of interest. Presence of “marketed to professionals” language triggers Medium confidence per rules.</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="b">
+          <t>Healthcare/medical facility with treatment rooms; no indication of nursery, SEN school, or food retail current or former use. Mention of adjacent Co-op is irrelevant. Contains suitability/variety language, so confidence is Medium.</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -773,23 +779,23 @@
           <t>HK-F002</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>SEN School</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Listing states it is currently let to and operated by an independent special educational needs provider and is currently operating as an SEN school with F1 consent and an active lease. Explicit current-use in target sector.</t>
+          <t>Currently operating as an independent special educational needs school with F1 (formerly D1) consent and dedicated SEN facilities (sensory/therapy suites).</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -803,14 +809,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Currently operating as a vape/e-cig retailer and a hairdressing salon with residential flats above; no childcare, SEN school, or food retail use, and explicitly no consent for childcare/education or food retail.</t>
+          <t>Two ground floor units let to a vape retailer and a hairdresser with A1/A2 consent; no current or former nursery, SEN, or food retail use or consent indicated.</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -830,16 +836,16 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Currently operating as a car showroom with residence; not a nursery, SEN school, or food store. “Suitable for” other uses does not affect classification without a named current tenant per rules.</t>
+          <t>Listing is a freehold car showroom with residence; no current or former use as nursery, SEN school, or food store. Only generic suitability for alternative uses is mentioned, which does not qualify for target sectors and triggers Medium confidence.</t>
         </is>
       </c>
       <c r="E16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -848,19 +854,19 @@
           <t>758763053880849.0</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Nursery</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Listing explicitly describes an operating children’s day nursery with Ofsted rating, staff, and current trading; no indications of vacancy or former use.</t>
+          <t>Currently operating children’s day nursery with Ofsted rating and registration for 75 children; explicitly a childcare facility.</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -873,22 +879,22 @@
           <t>88930830.0</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Nursery</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>The listing is offered with full vacant possession (“Vacant FREEHOLD Nursery Building”), which per Rule 2 signals None. Although it’s configured/operated as a nursery, the sale is on a vacant basis, so not currently operating for our purposes. Flagging Medium due to explicit nursery use/fit-out mentioned.</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="b">
+          <t>Explicitly a nursery building (“currently configured and operated as a Nursery (Use Class E)”) being sold with vacant possession. This is sector-relevant as a (vacant) nursery. Confidence set to Medium due to vacant status and alternative-use language in the listing.</t>
+        </is>
+      </c>
+      <c r="E18" t="b">
         <v>1</v>
       </c>
     </row>
@@ -903,17 +909,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>The listing is for airspace development rights to add residential units above an existing building. Although the ground floor is let to Sainsbury’s (a food store), Rule 5 requires classifying what is being sold (the airspace), not the underlying tenant. Hence None, flagged Medium due to development rights above a target-sector tenant.</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="b">
+          <t>Airspace development for residential apartments is being sold. Although the ground floor is let to Sainsbury’s (a food store), Rule 5 requires classifying what is being sold, not the tenant below. Therefore not acquisition-relevant to nursery/SEN/food store. Confidence Medium due to airspace above a target-sector tenant.</t>
+        </is>
+      </c>
+      <c r="E19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -930,16 +936,16 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Current use is an industrial/warehouse complex for manufacturing, storage, and distribution. No indication of operation as a nursery, SEN school, or food retail store; clearly unrelated to target sectors.</t>
+          <t>Industrial/warehouse complex with manufacturing and storage uses; no mention of current or former nursery, SEN school, or food store use. Generic “suitable for” language is present, so classify as None with Medium confidence.</t>
         </is>
       </c>
       <c r="E20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -948,22 +954,22 @@
           <t>88931949.0</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Nursery</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The listing is offered with full vacant possession (“Vacant FREEHOLD Nursery Building”), so it is not currently operating as a nursery. Despite nursery fit-out and sector wording, current use is vacant per rule 2.</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="b">
+          <t>Vacant freehold property currently configured and fitted out as a children’s nursery with play areas and nursery-specific features; marketed as a comprehensive nursery offering. Presence of “variety of future uses” language and vacant/former use triggers Medium confidence.</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -973,19 +979,19 @@
           <t>73143559</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Food Store</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>The listing states the unit is currently used as a small convenience store and is let on an ongoing lease with the business unaffected by the sale, indicating an operating food retail use.</t>
+          <t>The listing describes an operating convenience store (“open plan retail space used as a small convenience store”) with an ongoing lease and business unaffected. This is a current food retail use.</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -998,22 +1004,22 @@
           <t>HK-F003</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Nursery</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Currently vacant; description states “most recently trading as” and that the operator’s “lease expired,” which per rules signals None. D1 nursery consent and retained nursery fit-out/suitable-for language indicate former/potential use only, not current operation.</t>
-        </is>
-      </c>
-      <c r="E23" s="1" t="b">
+          <t>Vacant former children’s day nursery with D1 (nursery) consent and retained nursery-specific fit-out (low-level sinks, kitchen, enclosed play area). Clear former use as a nursery; marked Medium due to vacant/former use and planning-consent trigger.</t>
+        </is>
+      </c>
+      <c r="E23" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1023,22 +1029,22 @@
           <t>89908812.0</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Food Store</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Listing states “Former Costcutter supermarket” and “will be sold vacant with no lease,” so it is not currently operating. Former use was a food store, hence None with medium confidence due to prior sector use.</t>
-        </is>
-      </c>
-      <c r="E24" s="1" t="b">
+          <t>Explicitly described as a former Costcutter supermarket (food retail) now vacant, which qualifies as Food Store under former use. Presence of “suitable for a variety of alternative uses” also triggers Medium confidence per rules.</t>
+        </is>
+      </c>
+      <c r="E24" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: predict.py now outputs CSV with original columns alongside Excel
</commit_message>
<xml_diff>
--- a/results/listings_classified.xlsx
+++ b/results/listings_classified.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The listing is a former Co-op convenience store with retained food-retail fixtures (chillers, shelving) and is vacant, making it acquisition-relevant as a food retail property. Presence of former/vacant target-sector use triggers Medium confidence per rules.</t>
+          <t>Explicitly a former Co-op convenience store with retained chiller cabinets and shelving, indicating prior food retail use suitable for re-occupation by a food operator.</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -516,7 +516,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Listing is for an acre of ancient woodland/land with generic development potential; no current or former nursery, SEN school, or food store use or consent indicated. Generic opportunity language does not qualify under the rules.</t>
+          <t>Listing is a parcel of ancient woodland/land with speculative development potential and no mention of current or former nursery, SEN school, or food store use. Generic development language only; no sector-specific relevance.</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -541,7 +541,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Property is a fully let mixed-use investment with generic retail on ground/first floors and a dance studio on the second. No indication of current or former use as a nursery, SEN school, or food store, and no suitability/alternative-use language. Therefore not relevant to target sectors.</t>
+          <t>Fully let high-street investment comprising generic retail space with storage and a dance studio; no indication of nursery, SEN school, or food store current/former use or sector-specific fit-out/consent.</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -566,7 +566,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>The property is a former café with residential accommodation above and generic ‘variety of alternative uses’ language. There is no indication of current or former use as a nursery, SEN school, or food retail store. Nearby occupiers (e.g., Co-Op) are location context only. Suitability/alternative-use phrasing triggers Medium confidence per rules.</t>
+          <t>The property is a former café with residential accommodation and general alternative-use language. No indication of current or former use as a nursery, SEN school, or food store.</t>
         </is>
       </c>
       <c r="E5" t="b">
@@ -591,7 +591,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The property is a former doctor’s surgery with generic suitability language for various uses. There is no mention of a nursery, SEN school, or food store current or former use. Generic suitability phrases are present, triggering Medium confidence.</t>
+          <t>Former doctor’s surgery with generic ‘variety of alternative uses’ language; no mention of nursery, SEN school, or food store current or former use.</t>
         </is>
       </c>
       <c r="E6" t="b">
@@ -616,7 +616,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Property comprises a tanning shop with a flat above; no current or former nursery, SEN school, or food store use. Mention of a Budgens/Premier store is merely nearby (location context) and must be ignored per rules.</t>
+          <t>Subject property is a ground-floor sunbed/tanning shop with a flat above. No current or former nursery, SEN school, or food retail use is indicated. Mention of a nearby Budgens/Premier store refers to surrounding amenities, not the subject property.</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -641,7 +641,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mixed-use property with a retail shop (bath products) and a holiday apartment. No indication of current or former use as a nursery, SEN school, or food store. Includes suitability phrasing (“could be used for a new retail business”), triggering Medium confidence per rules.</t>
+          <t>Mixed-use property with a bath products retail shop and holiday apartment; no indication of nursery, SEN school, or food retail use. The phrase “could be used for a new retail business” introduces suitability language, triggering Medium confidence.</t>
         </is>
       </c>
       <c r="E8" t="b">
@@ -666,7 +666,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Listing is a Grade II listed freehouse pub with accommodation; no mention of nursery, SEN school, or food retail current or former use. Nearby schools are location context only.</t>
+          <t>Grade II listed public house (pub) with no mention of nursery, SEN school, or food retail use; no suitability/alternative-use language. Not relevant to target sectors.</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -691,7 +691,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A fully let multi-let industrial/trade park investment with trade counter units; no current or former nursery, SEN school, or food retail use indicated and no sector-specific fit-out or consent mentioned.</t>
+          <t>Listing is a fully let multi-let industrial/trade park investment with industrial/trade counter units. No current or former use as nursery, SEN school, or food store is indicated. Mentions of nearby occupiers are irrelevant per rules. Therefore not relevant to target sectors.</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -716,7 +716,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Industrial business sale for a fire door manufacturer/joinery with no indication of current or former use as a nursery, SEN school, or food store, nor any sector-specific planning or fit-out mentioned.</t>
+          <t>Industrial fire door manufacturing/joinery business for sale with no mention of nursery, SEN school, or food retail current or former use.</t>
         </is>
       </c>
       <c r="E11" t="b">
@@ -741,7 +741,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The listing is a mixed-use freehold investment comprising a workshop/garage and a separate retail shop sold off on a long lease. No mention of nursery, SEN school, or food retail use for the subject premises; references to Tesco Express are only nearby occupiers and must be ignored. Development/airspace notes do not relate to a target-sector tenant. Therefore, no meaningful connection to Nursery, SEN School, or Food Store.</t>
+          <t>Listing is a freehold investment with flats, a leased retail shop, and a leased workshop/garage plus airspace/redevelopment potential. No current or former use as nursery, SEN school, or food store is indicated. Mention of Tesco Express is only as a nearby occupier (to be ignored).</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -766,7 +766,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Healthcare/medical facility with treatment rooms; no indication of nursery, SEN school, or food retail current or former use. Mention of adjacent Co-op is irrelevant. Contains suitability/variety language, so confidence is Medium.</t>
+          <t>The listing is a healthcare/medical clinic space with treatment rooms; no current or former use as a nursery, SEN school, or food store is indicated. The mention of an adjacent Co‑Op is just location context. Marketing language to professionals and “variety” phrasing triggers Medium confidence per rules.</t>
         </is>
       </c>
       <c r="E13" t="b">
@@ -791,7 +791,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Currently operating as an independent special educational needs school with F1 (formerly D1) consent and dedicated SEN facilities (sensory/therapy suites).</t>
+          <t>Currently operating as an independent special educational needs school with F1 (formerly D1) consent, dedicated SEN facilities (sensory/therapy suites), and explicit sector use. Confidence marked Medium due to presence of planning consent language, which triggers Medium per rules.</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -816,7 +816,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Two ground floor units let to a vape retailer and a hairdresser with A1/A2 consent; no current or former nursery, SEN, or food retail use or consent indicated.</t>
+          <t>Ground-floor units let to a vape shop and hairdresser with no childcare/education or food retail use or consent. No former use in target sectors indicated. Listing is a generic mixed-use investment, not sector-relevant.</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -841,7 +841,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Listing is a freehold car showroom with residence; no current or former use as nursery, SEN school, or food store. Only generic suitability for alternative uses is mentioned, which does not qualify for target sectors and triggers Medium confidence.</t>
+          <t>Listing is a car showroom with residence and only generic suitability for various uses; no current or former nursery, SEN school, or food store use is indicated. Presence of “ideal for any variety of other uses” triggers Medium confidence per rules.</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -866,7 +866,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Currently operating children’s day nursery with Ofsted rating and registration for 75 children; explicitly a childcare facility.</t>
+          <t>Currently operating children’s day nursery with Ofsted rating and registered places; explicitly a childcare facility.</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -891,7 +891,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Explicitly a nursery building (“currently configured and operated as a Nursery (Use Class E)”) being sold with vacant possession. This is sector-relevant as a (vacant) nursery. Confidence set to Medium due to vacant status and alternative-use language in the listing.</t>
+          <t>Listing explicitly describes a freehold property configured and operated as a nursery being sold with vacant possession. This is directly relevant to the Nursery sector. Presence of “suitable for a range of uses” language triggers Medium confidence per rules.</t>
         </is>
       </c>
       <c r="E18" t="b">
@@ -916,7 +916,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Airspace development for residential apartments is being sold. Although the ground floor is let to Sainsbury’s (a food store), Rule 5 requires classifying what is being sold, not the tenant below. Therefore not acquisition-relevant to nursery/SEN/food store. Confidence Medium due to airspace above a target-sector tenant.</t>
+          <t>This is an airspace development sale to add three residential apartments. Although the ground floor is let to Sainsbury’s (a food store), Rule 5 applies—classify what is being sold (airspace/development rights), not the underlying tenant—so it does not qualify for Food Store. Confidence is Medium due to the explicit airspace-over-target-tenant trigger.</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -941,7 +941,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Industrial/warehouse complex with manufacturing and storage uses; no mention of current or former nursery, SEN school, or food store use. Generic “suitable for” language is present, so classify as None with Medium confidence.</t>
+          <t>Industrial/warehouse units with no mention of nursery, SEN school, or food retail current or former use. Only generic suitability language for industrial uses is present, which does not qualify any target sector.</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -966,7 +966,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Vacant freehold property currently configured and fitted out as a children’s nursery with play areas and nursery-specific features; marketed as a comprehensive nursery offering. Presence of “variety of future uses” language and vacant/former use triggers Medium confidence.</t>
+          <t>Vacant freehold building explicitly configured and fitted out as a children’s nursery, with dedicated play areas and nursery-specific features. Despite clarity, confidence is Medium due to vacant status and alternative-use language in the listing.</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -991,7 +991,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>The listing describes an operating convenience store (“open plan retail space used as a small convenience store”) with an ongoing lease and business unaffected. This is a current food retail use.</t>
+          <t>The listing states the unit is currently used as a small convenience store (food retail). No alternative-use or former-use ambiguity is present.</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Vacant former children’s day nursery with D1 (nursery) consent and retained nursery-specific fit-out (low-level sinks, kitchen, enclosed play area). Clear former use as a nursery; marked Medium due to vacant/former use and planning-consent trigger.</t>
+          <t>Vacant former children’s day nursery with D1 nursery consent and retained nursery-specific fit-out (low-level sinks, kitchen, secured outdoor play area); explicitly marketed for nursery/childcare use.</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Explicitly described as a former Costcutter supermarket (food retail) now vacant, which qualifies as Food Store under former use. Presence of “suitable for a variety of alternative uses” also triggers Medium confidence per rules.</t>
+          <t>Explicitly described as a former Costcutter supermarket (former food retail use). Although vacant and mentions suitability for alternative uses, it retains clear former food store identity.</t>
         </is>
       </c>
       <c r="E24" t="b">

</xml_diff>

<commit_message>
chore: regenerate results after removing requires_human_review
</commit_message>
<xml_diff>
--- a/results/listings_classified.xlsx
+++ b/results/listings_classified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,11 +467,6 @@
           <t>reasoning</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>requires_human_review</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -491,11 +486,8 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Explicitly a former Co-op convenience store with retained chiller cabinets and shelving, indicating prior food retail use suitable for re-occupation by a food operator.</t>
-        </is>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
+          <t>Specific former sector use stated: former Co-op convenience store, vacant, with retained food retail fit-out (chillers, shelving) and A1 use. This clearly aligns with food retail. Confidence set to Medium due to former/vacant status triggering the Medium rule.</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -516,11 +508,8 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Listing is a parcel of ancient woodland/land with speculative development potential and no mention of current or former nursery, SEN school, or food store use. Generic development language only; no sector-specific relevance.</t>
-        </is>
-      </c>
-      <c r="E3" t="b">
-        <v>0</v>
+          <t>Sale of an acre of ancient woodland/land with possible development potential; no current or former use or consent related to nursery, SEN school, or food retail.</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -541,11 +530,8 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Fully let high-street investment comprising generic retail space with storage and a dance studio; no indication of nursery, SEN school, or food store current/former use or sector-specific fit-out/consent.</t>
-        </is>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
+          <t>Listing is a fully-let high street investment with generic retail on ground/first floors and a dance studio on the second floor. No mention of nursery/SEN use or food retail (current or former).</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -566,11 +552,8 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>The property is a former café with residential accommodation and general alternative-use language. No indication of current or former use as a nursery, SEN school, or food store.</t>
-        </is>
-      </c>
-      <c r="E5" t="b">
-        <v>1</v>
+          <t>Property is a former café with mixed-use/residential elements and general redevelopment potential. No current or former use as nursery, SEN school, or food retail is indicated. Suitability/alternative-use language is present, triggering Medium confidence.</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -591,11 +574,8 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Former doctor’s surgery with generic ‘variety of alternative uses’ language; no mention of nursery, SEN school, or food store current or former use.</t>
-        </is>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
+          <t>Former doctor’s surgery with no mention of nursery, SEN school, or food retail use. The listing only includes generic suitability language for a variety of alternative uses, which does not qualify it for target sectors and triggers Medium confidence.</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -616,11 +596,8 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Subject property is a ground-floor sunbed/tanning shop with a flat above. No current or former nursery, SEN school, or food retail use is indicated. Mention of a nearby Budgens/Premier store refers to surrounding amenities, not the subject property.</t>
-        </is>
-      </c>
-      <c r="E7" t="b">
-        <v>0</v>
+          <t>Property comprises a tanning shop with a residential flat above. No current or former nursery, SEN school, or food store use. Mention of nearby Budgens/Premier is a location point, not the subject property.</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -641,11 +618,8 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mixed-use property with a bath products retail shop and holiday apartment; no indication of nursery, SEN school, or food retail use. The phrase “could be used for a new retail business” introduces suitability language, triggering Medium confidence.</t>
-        </is>
-      </c>
-      <c r="E8" t="b">
-        <v>1</v>
+          <t>Mixed-use property with a bath products retail shop/workshop and a holiday apartment; no indication of nursery, SEN school, or food retail use. Contains suitability/alternative-use style language about being used for a new retail business, triggering Medium confidence.</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -666,11 +640,8 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Grade II listed public house (pub) with no mention of nursery, SEN school, or food retail use; no suitability/alternative-use language. Not relevant to target sectors.</t>
-        </is>
-      </c>
-      <c r="E9" t="b">
-        <v>0</v>
+          <t>The listing is a Grade II listed public house (freehouse) with no mention of current or former use as a nursery, SEN school, or food store. No suitability/alternative-use language is present. Therefore it does not relate to the target sectors.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -691,11 +662,8 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Listing is a fully let multi-let industrial/trade park investment with industrial/trade counter units. No current or former use as nursery, SEN school, or food store is indicated. Mentions of nearby occupiers are irrelevant per rules. Therefore not relevant to target sectors.</t>
-        </is>
-      </c>
-      <c r="E10" t="b">
-        <v>0</v>
+          <t>Industrial/trade park investment with multiple industrial units; no mention of nursery, SEN school, or food retail current or former use, and no suitability/alternative-use language tied to those sectors.</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -716,11 +684,8 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Industrial fire door manufacturing/joinery business for sale with no mention of nursery, SEN school, or food retail current or former use.</t>
-        </is>
-      </c>
-      <c r="E11" t="b">
-        <v>0</v>
+          <t>Industrial business (fire door manufacturer/joinery) with no current or former use related to nurseries, SEN schools, or food retail, and no suitability/alternative-use language indicating relevance.</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -741,11 +706,8 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Listing is a freehold investment with flats, a leased retail shop, and a leased workshop/garage plus airspace/redevelopment potential. No current or former use as nursery, SEN school, or food store is indicated. Mention of Tesco Express is only as a nearby occupier (to be ignored).</t>
-        </is>
-      </c>
-      <c r="E12" t="b">
-        <v>0</v>
+          <t>Freehold/long-leasehold investment comprising flats, a garage/workshop, and a separate ground-floor retail unit on long lease. No mention of nursery, SEN school, or food store use (nearby Tesco is just a location reference). Development potential/airspace noted but not sector-specific.</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -766,11 +728,8 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The listing is a healthcare/medical clinic space with treatment rooms; no current or former use as a nursery, SEN school, or food store is indicated. The mention of an adjacent Co‑Op is just location context. Marketing language to professionals and “variety” phrasing triggers Medium confidence per rules.</t>
-        </is>
-      </c>
-      <c r="E13" t="b">
-        <v>1</v>
+          <t>Healthcare/medical treatment rooms and rehab space; no mention of nursery, SEN school, or food retail use. Reference to adjacent Co-Op is location only. Marketing uses suitability language and targets professionals, triggering Medium confidence.</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -791,11 +750,8 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Currently operating as an independent special educational needs school with F1 (formerly D1) consent, dedicated SEN facilities (sensory/therapy suites), and explicit sector use. Confidence marked Medium due to presence of planning consent language, which triggers Medium per rules.</t>
-        </is>
-      </c>
-      <c r="E14" t="b">
-        <v>1</v>
+          <t>Currently operated by a special educational needs provider with F1 (formerly D1) consent and SEN-specific facilities (sensory/therapy suites).</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -816,11 +772,8 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Ground-floor units let to a vape shop and hairdresser with no childcare/education or food retail use or consent. No former use in target sectors indicated. Listing is a generic mixed-use investment, not sector-relevant.</t>
-        </is>
-      </c>
-      <c r="E15" t="b">
-        <v>0</v>
+          <t>Mixed-use investment with ground-floor tenants as a vape shop and hairdresser; no current or former nursery/SEN/food retail use and explicitly no childcare/education or food retail consent. No sector-relevant fit-out or planning; no alternative-use language indicating target sectors.</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -841,11 +794,8 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Listing is a car showroom with residence and only generic suitability for various uses; no current or former nursery, SEN school, or food store use is indicated. Presence of “ideal for any variety of other uses” triggers Medium confidence per rules.</t>
-        </is>
-      </c>
-      <c r="E16" t="b">
-        <v>1</v>
+          <t>Listing is a car showroom with residence; mentions generic suitability for various uses but no current or former nursery, SEN school, or food store use. Presence of “suitable for/variety of uses” triggers Medium confidence.</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -866,11 +816,8 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Currently operating children’s day nursery with Ofsted rating and registered places; explicitly a childcare facility.</t>
-        </is>
-      </c>
-      <c r="E17" t="b">
-        <v>0</v>
+          <t>Currently operating children’s day nursery with Ofsted rating and business details; clearly a nursery asset.</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -891,11 +838,8 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Listing explicitly describes a freehold property configured and operated as a nursery being sold with vacant possession. This is directly relevant to the Nursery sector. Presence of “suitable for a range of uses” language triggers Medium confidence per rules.</t>
-        </is>
-      </c>
-      <c r="E18" t="b">
-        <v>1</v>
+          <t>Listing explicitly describes a vacant freehold nursery building currently configured/operated as a nursery and sold with vacant possession. This directly ties to the Nursery sector. Presence of “suitable for a range of uses” and vacant status triggers Medium confidence per rules.</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -916,11 +860,8 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>This is an airspace development sale to add three residential apartments. Although the ground floor is let to Sainsbury’s (a food store), Rule 5 applies—classify what is being sold (airspace/development rights), not the underlying tenant—so it does not qualify for Food Store. Confidence is Medium due to the explicit airspace-over-target-tenant trigger.</t>
-        </is>
-      </c>
-      <c r="E19" t="b">
-        <v>1</v>
+          <t>The listing sells airspace development rights to build residential apartments above a building whose ground floor is let to Sainsbury’s. Per Rule 5, classify what is being sold (airspace/residential), not the underlying food store tenant; therefore none of the target sectors apply. Confidence is Medium due to the specific trigger: airspace/development rights above a target-sector tenant.</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -941,11 +882,8 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Industrial/warehouse units with no mention of nursery, SEN school, or food retail current or former use. Only generic suitability language for industrial uses is present, which does not qualify any target sector.</t>
-        </is>
-      </c>
-      <c r="E20" t="b">
-        <v>1</v>
+          <t>Industrial/warehouse complex with generic suitability for manufacturing/storage/distribution; no current or former use as nursery, SEN school, or food store mentioned. Presence of “suitable for” language triggers Medium confidence.</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -966,11 +904,8 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Vacant freehold building explicitly configured and fitted out as a children’s nursery, with dedicated play areas and nursery-specific features. Despite clarity, confidence is Medium due to vacant status and alternative-use language in the listing.</t>
-        </is>
-      </c>
-      <c r="E21" t="b">
-        <v>1</v>
+          <t>Listing explicitly describes a vacant freehold children’s nursery building with sector-specific fit-out (enclosed play areas, configured for childcare). Vacant former/current nursery use qualifies as Nursery. Confidence is Medium due to vacant/former use and “variety of future uses” language.</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -991,11 +926,8 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>The listing states the unit is currently used as a small convenience store (food retail). No alternative-use or former-use ambiguity is present.</t>
-        </is>
-      </c>
-      <c r="E22" t="b">
-        <v>0</v>
+          <t>The listing describes a retail unit currently trading as a small convenience store, i.e., a food retail use. No suitability/alternative-use or former/vacant language is present.</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1016,11 +948,8 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Vacant former children’s day nursery with D1 nursery consent and retained nursery-specific fit-out (low-level sinks, kitchen, secured outdoor play area); explicitly marketed for nursery/childcare use.</t>
-        </is>
-      </c>
-      <c r="E23" t="b">
-        <v>1</v>
+          <t>Vacant unit with explicit D1 consent for a children’s day nursery, most recently operated as a nursery, and retains nursery-specific fit-out (low-level sinks, play area). Meets sector relevance; vacancy/suitability language triggers Medium confidence per rules.</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1041,11 +970,8 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Explicitly described as a former Costcutter supermarket (former food retail use). Although vacant and mentions suitability for alternative uses, it retains clear former food store identity.</t>
-        </is>
-      </c>
-      <c r="E24" t="b">
-        <v>1</v>
+          <t>Explicitly described as a former Costcutter supermarket (food retail) even though now vacant. Presence of “suitable for a variety of alternative uses” triggers Medium confidence per rules.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>